<commit_message>
Email Sequence 2 Complete
</commit_message>
<xml_diff>
--- a/manual/VALID_Roofing_Outreach_Leads.xlsx
+++ b/manual/VALID_Roofing_Outreach_Leads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khandpv1/Desktop/.AntiGrav/lead-gen/manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5576D51B-76EF-F243-B560-5CD96F418422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{701B68A7-D265-D74B-8353-BFA8280C2C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="760" windowWidth="34500" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="479">
   <si>
     <t>Roofs Plus</t>
   </si>
@@ -1435,6 +1435,42 @@
   </si>
   <si>
     <t>goodoneconstruction@gmail.com</t>
+  </si>
+  <si>
+    <t>FACEBOOK</t>
+  </si>
+  <si>
+    <t>NEXTDOOR</t>
+  </si>
+  <si>
+    <t>INSTAGRAM</t>
+  </si>
+  <si>
+    <t>MANTA</t>
+  </si>
+  <si>
+    <t>OTRUCKING</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Kansas City, MO</t>
+  </si>
+  <si>
+    <t>Poplar Bluff, MO</t>
+  </si>
+  <si>
+    <t>Bluffton, IN</t>
+  </si>
+  <si>
+    <t>Little Rock, AR</t>
+  </si>
+  <si>
+    <t>Berkeley Springs, WV</t>
+  </si>
+  <si>
+    <t>Amarillo, TX</t>
+  </si>
+  <si>
+    <t>OPEN</t>
   </si>
 </sst>
 </file>
@@ -1566,7 +1602,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1619,24 +1655,18 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1941,35 +1971,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:H106"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="35" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="29.6640625" style="12" customWidth="1"/>
-    <col min="6" max="6" width="38" customWidth="1"/>
-    <col min="8" max="8" width="34.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="35" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="7" width="29.6640625" style="12" customWidth="1"/>
+    <col min="8" max="8" width="38" customWidth="1"/>
+    <col min="10" max="10" width="34.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20"/>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-    </row>
-    <row r="2" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="18"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="22"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+    </row>
+    <row r="2" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="20"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
         <v>349</v>
       </c>
@@ -1980,16 +2014,20 @@
         <v>351</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="F3" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H3" s="1"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="16" t="s">
         <v>354</v>
       </c>
@@ -1999,17 +2037,21 @@
       <c r="C4" s="4" t="s">
         <v>356</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>357</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="F4" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>359</v>
       </c>
@@ -2020,16 +2062,20 @@
         <v>361</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="F5" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G5" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="16" t="s">
         <v>364</v>
       </c>
@@ -2039,35 +2085,45 @@
       <c r="C6" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>366</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="F6" s="5" t="s">
         <v>367</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G6" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
         <v>368</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="2" t="s">
+      <c r="B7" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C7" s="17" t="s">
         <v>369</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="F7" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G7" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H7" s="1"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="16" t="s">
         <v>372</v>
       </c>
@@ -2077,17 +2133,21 @@
       <c r="C8" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="F8" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G8" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="15" t="s">
         <v>377</v>
       </c>
@@ -2098,16 +2158,20 @@
         <v>379</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="F9" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G9" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H9" s="1"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="16" t="s">
         <v>382</v>
       </c>
@@ -2117,15 +2181,19 @@
       <c r="C10" s="5" t="s">
         <v>384</v>
       </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="22" t="s">
+      <c r="D10" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="5" t="s">
         <v>385</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G10" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="15" t="s">
         <v>386</v>
       </c>
@@ -2135,15 +2203,21 @@
       <c r="C11" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="D11" s="1"/>
-      <c r="E11" s="21" t="s">
+      <c r="D11" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E11" s="1"/>
+      <c r="F11" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G11" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="16" t="s">
         <v>390</v>
       </c>
@@ -2153,17 +2227,21 @@
       <c r="C12" s="4" t="s">
         <v>392</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="E12" s="22" t="s">
+      <c r="F12" s="5" t="s">
         <v>394</v>
       </c>
-      <c r="F12" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G12" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="15" t="s">
         <v>395</v>
       </c>
@@ -2174,16 +2252,20 @@
         <v>397</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="E13" s="21" t="s">
+      <c r="F13" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G13" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H13" s="1"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="16" t="s">
         <v>400</v>
       </c>
@@ -2193,17 +2275,21 @@
       <c r="C14" s="5" t="s">
         <v>402</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="E14" s="22" t="s">
+      <c r="F14" s="5" t="s">
         <v>404</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G14" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="15" t="s">
         <v>405</v>
       </c>
@@ -2213,15 +2299,19 @@
       <c r="C15" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="D15" s="1"/>
-      <c r="E15" s="21" t="s">
+      <c r="D15" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E15" s="1"/>
+      <c r="F15" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G15" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="16" t="s">
         <v>409</v>
       </c>
@@ -2231,15 +2321,19 @@
       <c r="C16" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="D16" s="3"/>
-      <c r="E16" s="22" t="s">
+      <c r="D16" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E16" s="3"/>
+      <c r="F16" s="5" t="s">
         <v>412</v>
       </c>
-      <c r="F16" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G16" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="15" t="s">
         <v>413</v>
       </c>
@@ -2249,15 +2343,19 @@
       <c r="C17" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="D17" s="1"/>
-      <c r="E17" s="21" t="s">
+      <c r="D17" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E17" s="1"/>
+      <c r="F17" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G17" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H17" s="1"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="16" t="s">
         <v>417</v>
       </c>
@@ -2267,15 +2365,21 @@
       <c r="C18" s="5" t="s">
         <v>419</v>
       </c>
-      <c r="D18" s="3"/>
-      <c r="E18" s="22" t="s">
+      <c r="D18" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E18" s="3"/>
+      <c r="F18" s="5" t="s">
         <v>420</v>
       </c>
-      <c r="F18" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G18" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="15" t="s">
         <v>421</v>
       </c>
@@ -2286,16 +2390,20 @@
         <v>423</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="E19" s="21" t="s">
+      <c r="F19" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G19" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H19" s="1"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="16" t="s">
         <v>426</v>
       </c>
@@ -2305,17 +2413,21 @@
       <c r="C20" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>429</v>
       </c>
-      <c r="E20" s="22" t="s">
+      <c r="F20" s="5" t="s">
         <v>430</v>
       </c>
-      <c r="F20" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G20" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H20" s="3"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="15" t="s">
         <v>431</v>
       </c>
@@ -2326,16 +2438,20 @@
         <v>433</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="E21" s="21" t="s">
+      <c r="F21" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G21" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H21" s="1"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="16" t="s">
         <v>436</v>
       </c>
@@ -2345,17 +2461,21 @@
       <c r="C22" s="4" t="s">
         <v>438</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>439</v>
       </c>
-      <c r="E22" s="22" t="s">
+      <c r="F22" s="5" t="s">
         <v>440</v>
       </c>
-      <c r="F22" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G22" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H22" s="3"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="15" t="s">
         <v>441</v>
       </c>
@@ -2366,16 +2486,22 @@
         <v>438</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="E23" s="21" t="s">
+      <c r="F23" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G23" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="16" t="s">
         <v>445</v>
       </c>
@@ -2385,17 +2511,21 @@
       <c r="C24" s="4" t="s">
         <v>447</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>448</v>
       </c>
-      <c r="E24" s="22" t="s">
+      <c r="F24" s="5" t="s">
         <v>449</v>
       </c>
-      <c r="F24" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G24" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H24" s="3"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="15" t="s">
         <v>450</v>
       </c>
@@ -2406,52 +2536,68 @@
         <v>451</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="E25" s="21" t="s">
+      <c r="F25" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G25" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H25" s="1"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
         <v>454</v>
       </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="5" t="s">
+      <c r="B26" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="C26" s="18" t="s">
         <v>455</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>456</v>
       </c>
-      <c r="E26" s="22" t="s">
+      <c r="F26" s="5" t="s">
         <v>457</v>
       </c>
-      <c r="F26" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G26" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H26" s="3"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="15" t="s">
         <v>458</v>
       </c>
-      <c r="B27" s="1"/>
-      <c r="C27" s="2" t="s">
+      <c r="B27" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C27" s="17" t="s">
         <v>459</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="E27" s="21" t="s">
+      <c r="F27" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="F27" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G27" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H27" s="1"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="16" t="s">
         <v>462</v>
       </c>
@@ -2461,17 +2607,23 @@
       <c r="C28" s="5" t="s">
         <v>464</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>465</v>
       </c>
-      <c r="E28" s="22" t="s">
+      <c r="F28" s="5" t="s">
         <v>466</v>
       </c>
-      <c r="F28" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G28" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="13" t="s">
         <v>0</v>
       </c>
@@ -2482,16 +2634,20 @@
         <v>2</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G29" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H29" s="7"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="14" t="s">
         <v>5</v>
       </c>
@@ -2501,17 +2657,21 @@
       <c r="C30" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="F30" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F30" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G30" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H30" s="3"/>
+    </row>
+    <row r="31" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="13" t="s">
         <v>10</v>
       </c>
@@ -2522,16 +2682,22 @@
         <v>12</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E31" s="11" t="s">
+      <c r="F31" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="F31" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G31" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="14" t="s">
         <v>15</v>
       </c>
@@ -2541,17 +2707,21 @@
       <c r="C32" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E32" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E32" s="10" t="s">
+      <c r="F32" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="F32" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G32" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H32" s="3"/>
+    </row>
+    <row r="33" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="13" t="s">
         <v>19</v>
       </c>
@@ -2562,16 +2732,20 @@
         <v>20</v>
       </c>
       <c r="D33" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E33" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="F33" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F33" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G33" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H33" s="7"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="14" t="s">
         <v>23</v>
       </c>
@@ -2581,17 +2755,21 @@
       <c r="C34" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="F34" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F34" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G34" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H34" s="3"/>
+    </row>
+    <row r="35" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="13" t="s">
         <v>28</v>
       </c>
@@ -2602,16 +2780,20 @@
         <v>29</v>
       </c>
       <c r="D35" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E35" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="F35" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F35" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G35" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H35" s="7"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="14" t="s">
         <v>32</v>
       </c>
@@ -2621,17 +2803,23 @@
       <c r="C36" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E36" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E36" s="10" t="s">
+      <c r="F36" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="F36" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G36" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="13" t="s">
         <v>37</v>
       </c>
@@ -2642,16 +2830,20 @@
         <v>39</v>
       </c>
       <c r="D37" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E37" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="F37" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F37" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G37" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H37" s="7"/>
+    </row>
+    <row r="38" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="13" t="s">
         <v>42</v>
       </c>
@@ -2662,16 +2854,22 @@
         <v>44</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E38" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E38" s="11" t="s">
+      <c r="F38" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="F38" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G38" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="14" t="s">
         <v>47</v>
       </c>
@@ -2681,17 +2879,21 @@
       <c r="C39" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E39" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E39" s="10" t="s">
+      <c r="F39" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="F39" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G39" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H39" s="3"/>
+    </row>
+    <row r="40" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="13" t="s">
         <v>51</v>
       </c>
@@ -2702,16 +2904,20 @@
         <v>53</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E40" s="2" t="s">
+      <c r="F40" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="F40" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G40" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H40" s="7"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="14" t="s">
         <v>56</v>
       </c>
@@ -2721,17 +2927,23 @@
       <c r="C41" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E41" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E41" s="10" t="s">
+      <c r="F41" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F41" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G41" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="14" t="s">
         <v>62</v>
       </c>
@@ -2741,17 +2953,21 @@
       <c r="C42" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="E42" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="F42" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="F42" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G42" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H42" s="3"/>
+    </row>
+    <row r="43" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="13" t="s">
         <v>66</v>
       </c>
@@ -2762,16 +2978,20 @@
         <v>68</v>
       </c>
       <c r="D43" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E43" s="11" t="s">
+      <c r="F43" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="F43" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G43" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H43" s="7"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="14" t="s">
         <v>71</v>
       </c>
@@ -2781,17 +3001,21 @@
       <c r="C44" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D44" s="3" t="s">
+      <c r="D44" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E44" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E44" s="5" t="s">
+      <c r="F44" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="F44" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G44" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H44" s="3"/>
+    </row>
+    <row r="45" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="13" t="s">
         <v>75</v>
       </c>
@@ -2802,16 +3026,20 @@
         <v>77</v>
       </c>
       <c r="D45" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E45" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="F45" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F45" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G45" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H45" s="7"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="14" t="s">
         <v>80</v>
       </c>
@@ -2821,17 +3049,21 @@
       <c r="C46" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="D46" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E46" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E46" s="5" t="s">
+      <c r="F46" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="F46" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G46" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H46" s="3"/>
+    </row>
+    <row r="47" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="13" t="s">
         <v>84</v>
       </c>
@@ -2842,16 +3074,22 @@
         <v>86</v>
       </c>
       <c r="D47" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E47" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="E47" s="11" t="s">
+      <c r="F47" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="F47" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G47" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H47" s="7" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" s="14" t="s">
         <v>89</v>
       </c>
@@ -2861,17 +3099,21 @@
       <c r="C48" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D48" s="3" t="s">
+      <c r="D48" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E48" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E48" s="10" t="s">
+      <c r="F48" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="F48" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G48" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H48" s="3"/>
+    </row>
+    <row r="49" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="13" t="s">
         <v>94</v>
       </c>
@@ -2882,16 +3124,22 @@
         <v>96</v>
       </c>
       <c r="D49" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E49" s="2" t="s">
+      <c r="F49" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="F49" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G49" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H49" s="7" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="14" t="s">
         <v>99</v>
       </c>
@@ -2901,17 +3149,21 @@
       <c r="C50" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D50" s="3" t="s">
+      <c r="D50" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E50" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E50" s="5" t="s">
+      <c r="F50" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="F50" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G50" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H50" s="3"/>
+    </row>
+    <row r="51" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="13" t="s">
         <v>103</v>
       </c>
@@ -2922,16 +3174,20 @@
         <v>105</v>
       </c>
       <c r="D51" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E51" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E51" s="2" t="s">
+      <c r="F51" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F51" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G51" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H51" s="7"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" s="14" t="s">
         <v>108</v>
       </c>
@@ -2941,17 +3197,21 @@
       <c r="C52" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="D52" s="3" t="s">
+      <c r="D52" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E52" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="E52" s="10" t="s">
+      <c r="F52" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="F52" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G52" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H52" s="3"/>
+    </row>
+    <row r="53" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="13" t="s">
         <v>113</v>
       </c>
@@ -2962,16 +3222,20 @@
         <v>114</v>
       </c>
       <c r="D53" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E53" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="E53" s="11" t="s">
+      <c r="F53" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="F53" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G53" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H53" s="7"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" s="14" t="s">
         <v>117</v>
       </c>
@@ -2981,17 +3245,21 @@
       <c r="C54" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="D54" s="3" t="s">
+      <c r="D54" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E54" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="E54" s="5" t="s">
+      <c r="F54" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="F54" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G54" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H54" s="3"/>
+    </row>
+    <row r="55" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="13" t="s">
         <v>122</v>
       </c>
@@ -3002,16 +3270,20 @@
         <v>123</v>
       </c>
       <c r="D55" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E55" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="E55" s="11" t="s">
+      <c r="F55" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="F55" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G55" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H55" s="7"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="14" t="s">
         <v>126</v>
       </c>
@@ -3021,17 +3293,23 @@
       <c r="C56" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="D56" s="3" t="s">
+      <c r="D56" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E56" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="E56" s="5" t="s">
+      <c r="F56" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="F56" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G56" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="13" t="s">
         <v>131</v>
       </c>
@@ -3042,16 +3320,20 @@
         <v>132</v>
       </c>
       <c r="D57" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E57" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E57" s="2" t="s">
+      <c r="F57" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="F57" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G57" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H57" s="7"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="14" t="s">
         <v>134</v>
       </c>
@@ -3061,17 +3343,23 @@
       <c r="C58" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="D58" s="3" t="s">
+      <c r="D58" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E58" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="E58" s="10" t="s">
+      <c r="F58" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="F58" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G58" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="13" t="s">
         <v>139</v>
       </c>
@@ -3082,16 +3370,20 @@
         <v>141</v>
       </c>
       <c r="D59" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E59" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E59" s="2" t="s">
+      <c r="F59" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F59" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G59" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H59" s="7"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
         <v>144</v>
       </c>
@@ -3101,17 +3393,21 @@
       <c r="C60" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="D60" s="3" t="s">
+      <c r="D60" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E60" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="E60" s="10" t="s">
+      <c r="F60" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="F60" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G60" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H60" s="3"/>
+    </row>
+    <row r="61" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="13" t="s">
         <v>148</v>
       </c>
@@ -3122,16 +3418,20 @@
         <v>150</v>
       </c>
       <c r="D61" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E61" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E61" s="2" t="s">
+      <c r="F61" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F61" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G61" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H61" s="7"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" s="14" t="s">
         <v>153</v>
       </c>
@@ -3141,17 +3441,21 @@
       <c r="C62" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="D62" s="3" t="s">
+      <c r="D62" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E62" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="E62" s="5" t="s">
+      <c r="F62" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="F62" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G62" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H62" s="3"/>
+    </row>
+    <row r="63" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" s="13" t="s">
         <v>158</v>
       </c>
@@ -3162,16 +3466,20 @@
         <v>159</v>
       </c>
       <c r="D63" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E63" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="E63" s="2" t="s">
+      <c r="F63" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F63" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G63" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H63" s="7"/>
+    </row>
+    <row r="64" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" s="13" t="s">
         <v>162</v>
       </c>
@@ -3182,16 +3490,20 @@
         <v>164</v>
       </c>
       <c r="D64" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E64" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="F64" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="F64" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G64" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H64" s="7"/>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="14" t="s">
         <v>167</v>
       </c>
@@ -3201,17 +3513,21 @@
       <c r="C65" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="D65" s="3" t="s">
+      <c r="D65" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E65" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="E65" s="10" t="s">
+      <c r="F65" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="F65" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G65" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H65" s="3"/>
+    </row>
+    <row r="66" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="13" t="s">
         <v>172</v>
       </c>
@@ -3222,16 +3538,20 @@
         <v>174</v>
       </c>
       <c r="D66" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E66" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="E66" s="2" t="s">
+      <c r="F66" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="F66" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G66" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H66" s="7"/>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="14" t="s">
         <v>177</v>
       </c>
@@ -3241,17 +3561,21 @@
       <c r="C67" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="D67" s="3" t="s">
+      <c r="D67" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E67" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="E67" s="10" t="s">
+      <c r="F67" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="F67" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G67" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H67" s="3"/>
+    </row>
+    <row r="68" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" s="13" t="s">
         <v>182</v>
       </c>
@@ -3262,16 +3586,20 @@
         <v>184</v>
       </c>
       <c r="D68" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="E68" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="E68" s="2" t="s">
+      <c r="F68" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="F68" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G68" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H68" s="7"/>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="14" t="s">
         <v>187</v>
       </c>
@@ -3281,17 +3609,21 @@
       <c r="C69" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="D69" s="3" t="s">
+      <c r="D69" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E69" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="E69" s="5" t="s">
+      <c r="F69" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="F69" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G69" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H69" s="3"/>
+    </row>
+    <row r="70" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" s="13" t="s">
         <v>191</v>
       </c>
@@ -3302,16 +3634,22 @@
         <v>193</v>
       </c>
       <c r="D70" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E70" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="E70" s="2" t="s">
+      <c r="F70" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="F70" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G70" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H70" s="7" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" s="14" t="s">
         <v>196</v>
       </c>
@@ -3321,17 +3659,21 @@
       <c r="C71" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="D71" s="8" t="s">
+      <c r="D71" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E71" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E71" s="5" t="s">
+      <c r="F71" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="F71" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G71" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H71" s="3"/>
+    </row>
+    <row r="72" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" s="13" t="s">
         <v>200</v>
       </c>
@@ -3342,16 +3684,20 @@
         <v>202</v>
       </c>
       <c r="D72" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E72" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="E72" s="2" t="s">
+      <c r="F72" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="F72" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G72" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H72" s="7"/>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" s="14" t="s">
         <v>205</v>
       </c>
@@ -3361,15 +3707,19 @@
       <c r="C73" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="D73" s="3"/>
-      <c r="E73" s="5" t="s">
+      <c r="D73" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E73" s="3"/>
+      <c r="F73" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="F73" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G73" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H73" s="3"/>
+    </row>
+    <row r="74" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A74" s="13" t="s">
         <v>209</v>
       </c>
@@ -3380,16 +3730,20 @@
         <v>211</v>
       </c>
       <c r="D74" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E74" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="E74" s="2" t="s">
+      <c r="F74" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="F74" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G74" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H74" s="7"/>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" s="14" t="s">
         <v>214</v>
       </c>
@@ -3399,15 +3753,19 @@
       <c r="C75" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D75" s="3"/>
-      <c r="E75" s="5" t="s">
+      <c r="D75" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E75" s="3"/>
+      <c r="F75" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="F75" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G75" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H75" s="3"/>
+    </row>
+    <row r="76" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" s="13" t="s">
         <v>218</v>
       </c>
@@ -3418,16 +3776,20 @@
         <v>219</v>
       </c>
       <c r="D76" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E76" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="E76" s="2" t="s">
+      <c r="F76" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="F76" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G76" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H76" s="7"/>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" s="14" t="s">
         <v>221</v>
       </c>
@@ -3437,17 +3799,23 @@
       <c r="C77" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="D77" s="3" t="s">
+      <c r="D77" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E77" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="E77" s="10" t="s">
+      <c r="F77" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="F77" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G77" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A78" s="13" t="s">
         <v>225</v>
       </c>
@@ -3458,16 +3826,22 @@
         <v>227</v>
       </c>
       <c r="D78" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E78" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="E78" s="11" t="s">
+      <c r="F78" s="11" t="s">
         <v>229</v>
       </c>
-      <c r="F78" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G78" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H78" s="7" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" s="14" t="s">
         <v>230</v>
       </c>
@@ -3477,17 +3851,21 @@
       <c r="C79" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="D79" s="3" t="s">
+      <c r="D79" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E79" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="E79" s="5" t="s">
+      <c r="F79" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="F79" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G79" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H79" s="3"/>
+    </row>
+    <row r="80" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A80" s="13" t="s">
         <v>235</v>
       </c>
@@ -3498,16 +3876,20 @@
         <v>237</v>
       </c>
       <c r="D80" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E80" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="E80" s="2" t="s">
+      <c r="F80" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="F80" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G80" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H80" s="7"/>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" s="14" t="s">
         <v>240</v>
       </c>
@@ -3517,17 +3899,23 @@
       <c r="C81" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="D81" s="3" t="s">
+      <c r="D81" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E81" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="E81" s="10" t="s">
+      <c r="F81" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="F81" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G81" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H81" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="13" t="s">
         <v>244</v>
       </c>
@@ -3538,16 +3926,20 @@
         <v>245</v>
       </c>
       <c r="D82" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E82" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="E82" s="2" t="s">
+      <c r="F82" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="F82" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G82" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H82" s="7"/>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" s="14" t="s">
         <v>248</v>
       </c>
@@ -3557,17 +3949,23 @@
       <c r="C83" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="D83" s="3" t="s">
+      <c r="D83" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E83" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="E83" s="5" t="s">
+      <c r="F83" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="F83" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G83" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H83" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A84" s="13" t="s">
         <v>253</v>
       </c>
@@ -3578,16 +3976,20 @@
         <v>255</v>
       </c>
       <c r="D84" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="E84" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="E84" s="2" t="s">
+      <c r="F84" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="F84" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G84" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H84" s="7"/>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="14" t="s">
         <v>258</v>
       </c>
@@ -3597,17 +3999,21 @@
       <c r="C85" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="D85" s="3" t="s">
+      <c r="D85" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E85" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="E85" s="5" t="s">
+      <c r="F85" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F85" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G85" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H85" s="3"/>
+    </row>
+    <row r="86" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A86" s="13" t="s">
         <v>103</v>
       </c>
@@ -3618,16 +4024,20 @@
         <v>260</v>
       </c>
       <c r="D86" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E86" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E86" s="2" t="s">
+      <c r="F86" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F86" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G86" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H86" s="7"/>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="14" t="s">
         <v>261</v>
       </c>
@@ -3637,17 +4047,21 @@
       <c r="C87" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="D87" s="3" t="s">
+      <c r="D87" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E87" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="E87" s="5" t="s">
+      <c r="F87" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="F87" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G87" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H87" s="3"/>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" s="14" t="s">
         <v>266</v>
       </c>
@@ -3657,17 +4071,21 @@
       <c r="C88" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="D88" s="3" t="s">
+      <c r="D88" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="E88" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="E88" s="10" t="s">
+      <c r="F88" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="F88" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G88" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H88" s="3"/>
+    </row>
+    <row r="89" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A89" s="13" t="s">
         <v>271</v>
       </c>
@@ -3678,16 +4096,20 @@
         <v>272</v>
       </c>
       <c r="D89" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="E89" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="E89" s="2" t="s">
+      <c r="F89" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="F89" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G89" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H89" s="7"/>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" s="14" t="s">
         <v>275</v>
       </c>
@@ -3697,17 +4119,21 @@
       <c r="C90" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="D90" s="3" t="s">
+      <c r="D90" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="E90" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="E90" s="5" t="s">
+      <c r="F90" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="F90" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G90" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H90" s="3"/>
+    </row>
+    <row r="91" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A91" s="13" t="s">
         <v>280</v>
       </c>
@@ -3718,34 +4144,48 @@
         <v>281</v>
       </c>
       <c r="D91" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E91" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="E91" s="2" t="s">
+      <c r="F91" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="F91" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G91" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H91" s="7" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="B92" s="3"/>
-      <c r="C92" s="4" t="s">
+      <c r="B92" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="C92" s="18" t="s">
         <v>285</v>
       </c>
-      <c r="D92" s="3" t="s">
+      <c r="D92" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="E92" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="E92" s="5" t="s">
+      <c r="F92" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="F92" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G92" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H92" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A93" s="13" t="s">
         <v>182</v>
       </c>
@@ -3756,16 +4196,20 @@
         <v>184</v>
       </c>
       <c r="D93" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="E93" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="E93" s="2" t="s">
+      <c r="F93" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="F93" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G93" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H93" s="7"/>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" s="14" t="s">
         <v>288</v>
       </c>
@@ -3775,17 +4219,21 @@
       <c r="C94" s="4" t="s">
         <v>289</v>
       </c>
-      <c r="D94" s="3" t="s">
+      <c r="D94" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E94" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="E94" s="5" t="s">
+      <c r="F94" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="F94" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G94" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H94" s="3"/>
+    </row>
+    <row r="95" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A95" s="13" t="s">
         <v>292</v>
       </c>
@@ -3796,34 +4244,44 @@
         <v>294</v>
       </c>
       <c r="D95" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E95" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="E95" s="2" t="s">
+      <c r="F95" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="F95" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G95" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H95" s="7"/>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A96" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="B96" s="3"/>
-      <c r="C96" s="4" t="s">
+      <c r="B96" s="19" t="s">
+        <v>476</v>
+      </c>
+      <c r="C96" s="18" t="s">
         <v>298</v>
       </c>
-      <c r="D96" s="3" t="s">
+      <c r="D96" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E96" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="E96" s="5" t="s">
+      <c r="F96" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="F96" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G96" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H96" s="3"/>
+    </row>
+    <row r="97" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A97" s="13" t="s">
         <v>301</v>
       </c>
@@ -3834,52 +4292,70 @@
         <v>303</v>
       </c>
       <c r="D97" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E97" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="E97" s="2" t="s">
+      <c r="F97" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F97" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G97" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H97" s="7"/>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="B98" s="3"/>
-      <c r="C98" s="4" t="s">
+      <c r="B98" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C98" s="18" t="s">
         <v>307</v>
       </c>
-      <c r="D98" s="3" t="s">
+      <c r="D98" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E98" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="E98" s="5" t="s">
+      <c r="F98" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="F98" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G98" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H98" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A99" s="13" t="s">
         <v>310</v>
       </c>
-      <c r="B99" s="1"/>
-      <c r="C99" s="9" t="s">
+      <c r="B99" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="C99" s="17" t="s">
         <v>311</v>
       </c>
       <c r="D99" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E99" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="E99" s="2" t="s">
+      <c r="F99" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="F99" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G99" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H99" s="7"/>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A100" s="14" t="s">
         <v>314</v>
       </c>
@@ -3889,17 +4365,23 @@
       <c r="C100" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="D100" s="3" t="s">
+      <c r="D100" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E100" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="E100" s="5" t="s">
+      <c r="F100" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="F100" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G100" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H100" s="3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A101" s="15" t="s">
         <v>321</v>
       </c>
@@ -3910,16 +4392,20 @@
         <v>323</v>
       </c>
       <c r="D101" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E101" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="E101" s="23" t="s">
+      <c r="F101" s="17" t="s">
         <v>325</v>
       </c>
-      <c r="F101" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G101" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H101" s="7"/>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A102" s="16" t="s">
         <v>326</v>
       </c>
@@ -3929,17 +4415,21 @@
       <c r="C102" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="D102" s="3" t="s">
+      <c r="D102" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E102" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="E102" s="24" t="s">
+      <c r="F102" s="18" t="s">
         <v>329</v>
       </c>
-      <c r="F102" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G102" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H102" s="3"/>
+    </row>
+    <row r="103" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A103" s="15" t="s">
         <v>330</v>
       </c>
@@ -3950,16 +4440,22 @@
         <v>332</v>
       </c>
       <c r="D103" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E103" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="E103" s="17" t="s">
+      <c r="F103" s="17" t="s">
         <v>334</v>
       </c>
-      <c r="F103" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G103" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="H103" s="7" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A104" s="16" t="s">
         <v>335</v>
       </c>
@@ -3969,17 +4465,21 @@
       <c r="C104" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="D104" s="3" t="s">
+      <c r="D104" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E104" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="E104" s="24" t="s">
+      <c r="F104" s="18" t="s">
         <v>339</v>
       </c>
-      <c r="F104" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G104" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H104" s="3"/>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A105" s="15" t="s">
         <v>340</v>
       </c>
@@ -3990,16 +4490,20 @@
         <v>341</v>
       </c>
       <c r="D105" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E105" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="E105" s="23" t="s">
+      <c r="F105" s="17" t="s">
         <v>343</v>
       </c>
-      <c r="F105" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G105" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H105" s="1"/>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A106" s="16" t="s">
         <v>344</v>
       </c>
@@ -4009,20 +4513,24 @@
       <c r="C106" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="D106" s="3" t="s">
+      <c r="D106" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="E106" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="E106" s="24" t="s">
+      <c r="F106" s="18" t="s">
         <v>347</v>
       </c>
-      <c r="F106" s="3" t="s">
-        <v>319</v>
-      </c>
+      <c r="G106" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H106" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C29" r:id="rId1" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
@@ -4069,89 +4577,93 @@
     <hyperlink ref="C26" r:id="rId42" xr:uid="{30448CFA-8DFC-CF49-B2EC-9F61F3E503F8}"/>
     <hyperlink ref="C27" r:id="rId43" xr:uid="{8B12F9FF-F77A-6942-9564-4B6F4EB56E38}"/>
     <hyperlink ref="C28" r:id="rId44" xr:uid="{6AC65864-4261-DD45-9793-98637E6BC331}"/>
-    <hyperlink ref="E29" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="E33" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="E34" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="E35" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="E37" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="E40" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="E42" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="E44" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="E45" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="E46" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="E49" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="E50" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="E51" r:id="rId57" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="E54" r:id="rId58" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="E56" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="E57" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="E59" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="E61" r:id="rId62" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="E62" r:id="rId63" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="E63" r:id="rId64" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="E64" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="E66" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="E68" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="E69" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="E70" r:id="rId69" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="E71" r:id="rId70" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="E72" r:id="rId71" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="E73" r:id="rId72" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="E74" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="E75" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
-    <hyperlink ref="E76" r:id="rId75" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
-    <hyperlink ref="E79" r:id="rId76" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
-    <hyperlink ref="E80" r:id="rId77" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
-    <hyperlink ref="E82" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
-    <hyperlink ref="E83" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
-    <hyperlink ref="E84" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
-    <hyperlink ref="E85" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
-    <hyperlink ref="E86" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
-    <hyperlink ref="E87" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
-    <hyperlink ref="E89" r:id="rId84" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
-    <hyperlink ref="E90" r:id="rId85" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
-    <hyperlink ref="E91" r:id="rId86" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
-    <hyperlink ref="E92" r:id="rId87" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
-    <hyperlink ref="E93" r:id="rId88" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
-    <hyperlink ref="E94" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
-    <hyperlink ref="E95" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
-    <hyperlink ref="E96" r:id="rId91" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
-    <hyperlink ref="E97" r:id="rId92" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
-    <hyperlink ref="E98" r:id="rId93" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
-    <hyperlink ref="E99" r:id="rId94" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
-    <hyperlink ref="E100" r:id="rId95" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
-    <hyperlink ref="E101" r:id="rId96" xr:uid="{AF74E925-77C5-DE4B-8120-BADC09997F11}"/>
-    <hyperlink ref="E102" r:id="rId97" xr:uid="{3EA834B2-28DE-6D4B-900F-CF837B70DAC9}"/>
-    <hyperlink ref="E103" r:id="rId98" xr:uid="{076EEC32-3BEF-EE4A-96DE-2634BCDAB59D}"/>
-    <hyperlink ref="E104" r:id="rId99" xr:uid="{F856EB8E-3A36-9C43-8D3C-4E1028370810}"/>
-    <hyperlink ref="E105" r:id="rId100" xr:uid="{46220F03-158A-0244-A2D4-5D0061826243}"/>
-    <hyperlink ref="E106" r:id="rId101" xr:uid="{68E2DF56-B313-AD4C-84FE-B2FD5CC6A92B}"/>
-    <hyperlink ref="E3" r:id="rId102" xr:uid="{1F273E6E-4DFE-A14D-89FE-FB34D81FEA52}"/>
-    <hyperlink ref="E4" r:id="rId103" xr:uid="{4B720C8A-EFC3-774F-A69F-94EDBC03D6CA}"/>
-    <hyperlink ref="E5" r:id="rId104" xr:uid="{3E992711-4A44-E849-B3A2-43C880ECF634}"/>
-    <hyperlink ref="E6" r:id="rId105" xr:uid="{98231305-6C44-744F-BB3D-13D9E8A3E562}"/>
-    <hyperlink ref="E7" r:id="rId106" xr:uid="{522AE97A-7375-C241-8E77-40A5035B87FC}"/>
-    <hyperlink ref="E8" r:id="rId107" xr:uid="{2FF5CB95-4209-2F44-AA08-E922691F6ECA}"/>
-    <hyperlink ref="E9" r:id="rId108" xr:uid="{D2B0E98C-29FD-504E-B472-E7E51973F900}"/>
-    <hyperlink ref="E10" r:id="rId109" xr:uid="{3CBA5D47-B563-A148-9FE1-FC84E2737C29}"/>
-    <hyperlink ref="E11" r:id="rId110" xr:uid="{CDA4B8F9-4A0C-7E47-A97E-14F1EE09A92A}"/>
-    <hyperlink ref="E12" r:id="rId111" xr:uid="{8367E3A8-E83D-554D-8FDA-09DA7DAC2847}"/>
-    <hyperlink ref="E13" r:id="rId112" xr:uid="{692976D2-190B-8C4E-9EF8-9C8DAB5F335C}"/>
-    <hyperlink ref="E14" r:id="rId113" xr:uid="{47DB8A04-8616-A049-8332-3449E9CF3EEE}"/>
-    <hyperlink ref="E15" r:id="rId114" xr:uid="{88051FD0-8E29-AD45-9108-C25A091D5178}"/>
-    <hyperlink ref="E16" r:id="rId115" xr:uid="{A7D4B439-11B6-D848-9C09-71C2A2D55AEE}"/>
-    <hyperlink ref="E17" r:id="rId116" xr:uid="{9F19F137-CFD5-4A47-A317-38DF4A8212C1}"/>
-    <hyperlink ref="E18" r:id="rId117" xr:uid="{04FEBF75-2C5A-554F-A26B-3D6D3DDBF08E}"/>
-    <hyperlink ref="E19" r:id="rId118" xr:uid="{F96A7F40-9C38-EF41-88EC-55F3FC272F5E}"/>
-    <hyperlink ref="E20" r:id="rId119" xr:uid="{2779D812-2C5A-0E41-BE9B-9B34CEAC1246}"/>
-    <hyperlink ref="E21" r:id="rId120" xr:uid="{A2B4D2A7-3F6F-D240-BA65-ABB9F9FC9546}"/>
-    <hyperlink ref="E22" r:id="rId121" xr:uid="{7DC7062B-B79F-9145-BEC7-86D533114158}"/>
-    <hyperlink ref="E23" r:id="rId122" xr:uid="{56FEB712-79BD-5840-A3D2-D5A2A7D8CF41}"/>
-    <hyperlink ref="E24" r:id="rId123" xr:uid="{96A0D1DD-B5C2-CD4D-B211-03888658F123}"/>
-    <hyperlink ref="E25" r:id="rId124" xr:uid="{D26CACAD-1965-C147-9EF1-6776332897F3}"/>
-    <hyperlink ref="E26" r:id="rId125" xr:uid="{F49AF5FE-8E63-4846-9C0D-135ED6B2143A}"/>
-    <hyperlink ref="E27" r:id="rId126" xr:uid="{2ADD6954-12F2-5447-8EA7-531C99FCE04F}"/>
-    <hyperlink ref="E28" r:id="rId127" xr:uid="{6957A36C-D524-B441-81E7-553ECAC9E224}"/>
+    <hyperlink ref="F29" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="F33" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="F34" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="F35" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="F37" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="F40" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="F42" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="F44" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="F45" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="F46" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="F49" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="F50" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="F51" r:id="rId57" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="F54" r:id="rId58" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="F56" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="F57" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="F59" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="F61" r:id="rId62" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="F62" r:id="rId63" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="F63" r:id="rId64" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="F64" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="F66" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="F68" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="F69" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="F70" r:id="rId69" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="F71" r:id="rId70" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="F72" r:id="rId71" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="F73" r:id="rId72" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="F74" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="F75" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="F76" r:id="rId75" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="F79" r:id="rId76" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="F80" r:id="rId77" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="F82" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="F83" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="F84" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="F85" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="F86" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="F87" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
+    <hyperlink ref="F89" r:id="rId84" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
+    <hyperlink ref="F90" r:id="rId85" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
+    <hyperlink ref="F91" r:id="rId86" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
+    <hyperlink ref="F92" r:id="rId87" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="F93" r:id="rId88" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
+    <hyperlink ref="F94" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
+    <hyperlink ref="F95" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
+    <hyperlink ref="F96" r:id="rId91" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
+    <hyperlink ref="F97" r:id="rId92" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
+    <hyperlink ref="F98" r:id="rId93" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
+    <hyperlink ref="F99" r:id="rId94" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
+    <hyperlink ref="F100" r:id="rId95" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
+    <hyperlink ref="F101" r:id="rId96" xr:uid="{AF74E925-77C5-DE4B-8120-BADC09997F11}"/>
+    <hyperlink ref="F102" r:id="rId97" xr:uid="{3EA834B2-28DE-6D4B-900F-CF837B70DAC9}"/>
+    <hyperlink ref="F103" r:id="rId98" xr:uid="{076EEC32-3BEF-EE4A-96DE-2634BCDAB59D}"/>
+    <hyperlink ref="F104" r:id="rId99" xr:uid="{F856EB8E-3A36-9C43-8D3C-4E1028370810}"/>
+    <hyperlink ref="F105" r:id="rId100" xr:uid="{46220F03-158A-0244-A2D4-5D0061826243}"/>
+    <hyperlink ref="F106" r:id="rId101" xr:uid="{68E2DF56-B313-AD4C-84FE-B2FD5CC6A92B}"/>
+    <hyperlink ref="F3" r:id="rId102" xr:uid="{1F273E6E-4DFE-A14D-89FE-FB34D81FEA52}"/>
+    <hyperlink ref="F4" r:id="rId103" xr:uid="{4B720C8A-EFC3-774F-A69F-94EDBC03D6CA}"/>
+    <hyperlink ref="F5" r:id="rId104" xr:uid="{3E992711-4A44-E849-B3A2-43C880ECF634}"/>
+    <hyperlink ref="F6" r:id="rId105" xr:uid="{98231305-6C44-744F-BB3D-13D9E8A3E562}"/>
+    <hyperlink ref="F7" r:id="rId106" xr:uid="{522AE97A-7375-C241-8E77-40A5035B87FC}"/>
+    <hyperlink ref="F8" r:id="rId107" xr:uid="{2FF5CB95-4209-2F44-AA08-E922691F6ECA}"/>
+    <hyperlink ref="F9" r:id="rId108" xr:uid="{D2B0E98C-29FD-504E-B472-E7E51973F900}"/>
+    <hyperlink ref="F10" r:id="rId109" xr:uid="{3CBA5D47-B563-A148-9FE1-FC84E2737C29}"/>
+    <hyperlink ref="F11" r:id="rId110" xr:uid="{CDA4B8F9-4A0C-7E47-A97E-14F1EE09A92A}"/>
+    <hyperlink ref="F12" r:id="rId111" xr:uid="{8367E3A8-E83D-554D-8FDA-09DA7DAC2847}"/>
+    <hyperlink ref="F13" r:id="rId112" xr:uid="{692976D2-190B-8C4E-9EF8-9C8DAB5F335C}"/>
+    <hyperlink ref="F14" r:id="rId113" xr:uid="{47DB8A04-8616-A049-8332-3449E9CF3EEE}"/>
+    <hyperlink ref="F15" r:id="rId114" xr:uid="{88051FD0-8E29-AD45-9108-C25A091D5178}"/>
+    <hyperlink ref="F16" r:id="rId115" xr:uid="{A7D4B439-11B6-D848-9C09-71C2A2D55AEE}"/>
+    <hyperlink ref="F17" r:id="rId116" xr:uid="{9F19F137-CFD5-4A47-A317-38DF4A8212C1}"/>
+    <hyperlink ref="F18" r:id="rId117" xr:uid="{04FEBF75-2C5A-554F-A26B-3D6D3DDBF08E}"/>
+    <hyperlink ref="F19" r:id="rId118" xr:uid="{F96A7F40-9C38-EF41-88EC-55F3FC272F5E}"/>
+    <hyperlink ref="F20" r:id="rId119" xr:uid="{2779D812-2C5A-0E41-BE9B-9B34CEAC1246}"/>
+    <hyperlink ref="F21" r:id="rId120" xr:uid="{A2B4D2A7-3F6F-D240-BA65-ABB9F9FC9546}"/>
+    <hyperlink ref="F22" r:id="rId121" xr:uid="{7DC7062B-B79F-9145-BEC7-86D533114158}"/>
+    <hyperlink ref="F23" r:id="rId122" xr:uid="{56FEB712-79BD-5840-A3D2-D5A2A7D8CF41}"/>
+    <hyperlink ref="F24" r:id="rId123" xr:uid="{96A0D1DD-B5C2-CD4D-B211-03888658F123}"/>
+    <hyperlink ref="F25" r:id="rId124" xr:uid="{D26CACAD-1965-C147-9EF1-6776332897F3}"/>
+    <hyperlink ref="F26" r:id="rId125" xr:uid="{F49AF5FE-8E63-4846-9C0D-135ED6B2143A}"/>
+    <hyperlink ref="F27" r:id="rId126" xr:uid="{2ADD6954-12F2-5447-8EA7-531C99FCE04F}"/>
+    <hyperlink ref="F28" r:id="rId127" xr:uid="{6957A36C-D524-B441-81E7-553ECAC9E224}"/>
+    <hyperlink ref="C92" r:id="rId128" xr:uid="{A70682D3-E195-AE4F-9087-CC83C617800F}"/>
+    <hyperlink ref="C96" r:id="rId129" xr:uid="{1EE13C88-C598-6647-AE88-7A784810E939}"/>
+    <hyperlink ref="C98" r:id="rId130" xr:uid="{DB8FCF4F-0F40-534F-ACE5-CDA9FE34390B}"/>
+    <hyperlink ref="C99" r:id="rId131" xr:uid="{BEE8D83E-AC2E-0C4E-B248-179F1CD9424B}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Email Sequence 3 Complete
</commit_message>
<xml_diff>
--- a/manual/VALID_Roofing_Outreach_Leads.xlsx
+++ b/manual/VALID_Roofing_Outreach_Leads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khandpv1/Desktop/.AntiGrav/lead-gen/manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{701B68A7-D265-D74B-8353-BFA8280C2C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5657C881-04CD-D74C-8431-210E71967208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="760" windowWidth="34500" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="480">
   <si>
     <t>Roofs Plus</t>
   </si>
@@ -1182,9 +1182,6 @@
     <t>austinandsonsconstruction@gmail.com</t>
   </si>
   <si>
-    <t>Jake</t>
-  </si>
-  <si>
     <t>Southern, CO</t>
   </si>
   <si>
@@ -1471,6 +1468,12 @@
   </si>
   <si>
     <t>OPEN</t>
+  </si>
+  <si>
+    <t>INVALID</t>
+  </si>
+  <si>
+    <t>Davis Construction Inc.</t>
   </si>
 </sst>
 </file>
@@ -1971,19 +1974,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="4" width="35" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="7" width="29.6640625" style="12" customWidth="1"/>
-    <col min="8" max="8" width="38" customWidth="1"/>
-    <col min="10" max="10" width="34.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="29.6640625" style="12" customWidth="1"/>
+    <col min="9" max="10" width="16.6640625" customWidth="1"/>
+    <col min="12" max="12" width="34.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="22"/>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
@@ -1992,8 +1995,10 @@
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
       <c r="H1" s="21"/>
-    </row>
-    <row r="2" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+    </row>
+    <row r="2" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="20"/>
       <c r="B2" s="21"/>
       <c r="C2" s="21"/>
@@ -2002,8 +2007,10 @@
       <c r="F2" s="21"/>
       <c r="G2" s="21"/>
       <c r="H2" s="21"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
         <v>349</v>
       </c>
@@ -2014,7 +2021,7 @@
         <v>351</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>352</v>
@@ -2026,8 +2033,10 @@
         <v>319</v>
       </c>
       <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="16" t="s">
         <v>354</v>
       </c>
@@ -2038,7 +2047,7 @@
         <v>356</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>357</v>
@@ -2049,9 +2058,13 @@
       <c r="G4" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H4" s="3"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H4" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>359</v>
       </c>
@@ -2062,7 +2075,7 @@
         <v>361</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>362</v>
@@ -2074,8 +2087,10 @@
         <v>319</v>
       </c>
       <c r="H5" s="1"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="16" t="s">
         <v>364</v>
       </c>
@@ -2086,7 +2101,7 @@
         <v>365</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>366</v>
@@ -2098,19 +2113,21 @@
         <v>319</v>
       </c>
       <c r="H6" s="3"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
         <v>368</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>369</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>370</v>
@@ -2122,8 +2139,12 @@
         <v>319</v>
       </c>
       <c r="H7" s="1"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I7" s="1"/>
+      <c r="J7" s="1" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="16" t="s">
         <v>372</v>
       </c>
@@ -2134,7 +2155,7 @@
         <v>374</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>375</v>
@@ -2145,9 +2166,13 @@
       <c r="G8" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H8" s="3"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H8" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="15" t="s">
         <v>377</v>
       </c>
@@ -2158,7 +2183,7 @@
         <v>379</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>380</v>
@@ -2170,460 +2195,508 @@
         <v>319</v>
       </c>
       <c r="H9" s="1"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="16" t="s">
+        <v>479</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="5" t="s">
         <v>383</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>384</v>
-      </c>
       <c r="D10" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" s="15" t="s">
         <v>385</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="H10" s="3"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="15" t="s">
+      <c r="B11" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>388</v>
-      </c>
       <c r="D11" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" s="16" t="s">
         <v>389</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="16" t="s">
+      <c r="B12" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>391</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>392</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="F12" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" s="15" t="s">
+        <v>394</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>394</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="15" t="s">
-        <v>395</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>396</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="E13" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" s="16" t="s">
         <v>399</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="H13" s="1"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
+      <c r="B14" s="3" t="s">
         <v>400</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="C14" s="5" t="s">
         <v>401</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>402</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="5" t="s">
         <v>403</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="G14" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" s="15" t="s">
         <v>404</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="H14" s="3"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="15" t="s">
+      <c r="B15" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>407</v>
-      </c>
       <c r="D15" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" s="16" t="s">
         <v>408</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="H15" s="1"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="16" t="s">
+      <c r="B16" s="3" t="s">
         <v>409</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" s="5" t="s">
         <v>410</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>411</v>
-      </c>
       <c r="D16" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" s="15" t="s">
         <v>412</v>
       </c>
-      <c r="G16" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="H16" s="3"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="15" t="s">
+      <c r="B17" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>415</v>
-      </c>
       <c r="D17" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18" s="16" t="s">
         <v>416</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="H17" s="1"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="16" t="s">
+      <c r="B18" s="3" t="s">
         <v>417</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="C18" s="5" t="s">
         <v>418</v>
       </c>
-      <c r="C18" s="5" t="s">
-        <v>419</v>
-      </c>
       <c r="D18" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A19" s="15" t="s">
         <v>420</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="15" t="s">
+      <c r="B19" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="D19" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="F19" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A21" s="15" t="s">
+        <v>430</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A22" s="16" t="s">
+        <v>435</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A23" s="15" t="s">
+        <v>440</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="J23" s="1"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A24" s="16" t="s">
+        <v>444</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" s="15" t="s">
+        <v>449</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" s="16" t="s">
+        <v>453</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>454</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" s="15" t="s">
+        <v>457</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>458</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="H19" s="1"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="16" t="s">
-        <v>426</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>427</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>428</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>430</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="H20" s="3"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="15" t="s">
-        <v>431</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>432</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="H21" s="1"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="16" t="s">
-        <v>436</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>437</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>468</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>439</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>440</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="H22" s="3"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="15" t="s">
-        <v>441</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="16" t="s">
-        <v>445</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>446</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>447</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>448</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>449</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="H24" s="3"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="15" t="s">
-        <v>450</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>451</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="H25" s="1"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="16" t="s">
-        <v>454</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>473</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>455</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>456</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>457</v>
-      </c>
-      <c r="G26" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="H26" s="3"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="15" t="s">
-        <v>458</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="C27" s="17" t="s">
+      <c r="E27" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>469</v>
-      </c>
-      <c r="E27" s="1" t="s">
+      <c r="F27" s="2" t="s">
         <v>460</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="G27" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28" s="16" t="s">
         <v>461</v>
       </c>
-      <c r="G27" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="H27" s="1"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" s="16" t="s">
+      <c r="B28" s="3" t="s">
         <v>462</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="C28" s="5" t="s">
         <v>463</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="D28" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>464</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="E28" s="3" t="s">
+      <c r="F28" s="5" t="s">
         <v>465</v>
       </c>
-      <c r="F28" s="5" t="s">
-        <v>466</v>
-      </c>
       <c r="G28" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H28" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H28" s="3"/>
+      <c r="I28" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J28" s="3"/>
+    </row>
+    <row r="29" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="13" t="s">
         <v>0</v>
       </c>
@@ -2634,7 +2707,7 @@
         <v>2</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>3</v>
@@ -2646,8 +2719,10 @@
         <v>319</v>
       </c>
       <c r="H29" s="7"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I29" s="7"/>
+      <c r="J29" s="7"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="14" t="s">
         <v>5</v>
       </c>
@@ -2658,7 +2733,7 @@
         <v>7</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>8</v>
@@ -2670,8 +2745,10 @@
         <v>319</v>
       </c>
       <c r="H30" s="3"/>
-    </row>
-    <row r="31" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+    </row>
+    <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="13" t="s">
         <v>10</v>
       </c>
@@ -2682,7 +2759,7 @@
         <v>12</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>13</v>
@@ -2693,11 +2770,15 @@
       <c r="G31" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H31" s="7" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H31" s="7"/>
+      <c r="I31" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="J31" s="7" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="14" t="s">
         <v>15</v>
       </c>
@@ -2708,7 +2789,7 @@
         <v>16</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>17</v>
@@ -2720,8 +2801,10 @@
         <v>319</v>
       </c>
       <c r="H32" s="3"/>
-    </row>
-    <row r="33" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+    </row>
+    <row r="33" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="13" t="s">
         <v>19</v>
       </c>
@@ -2732,7 +2815,7 @@
         <v>20</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>21</v>
@@ -2743,9 +2826,13 @@
       <c r="G33" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H33" s="7"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H33" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="I33" s="7"/>
+      <c r="J33" s="7"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="14" t="s">
         <v>23</v>
       </c>
@@ -2756,7 +2843,7 @@
         <v>25</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>26</v>
@@ -2768,8 +2855,10 @@
         <v>319</v>
       </c>
       <c r="H34" s="3"/>
-    </row>
-    <row r="35" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+    </row>
+    <row r="35" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="13" t="s">
         <v>28</v>
       </c>
@@ -2780,7 +2869,7 @@
         <v>29</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>30</v>
@@ -2792,8 +2881,10 @@
         <v>319</v>
       </c>
       <c r="H35" s="7"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="14" t="s">
         <v>32</v>
       </c>
@@ -2804,7 +2895,7 @@
         <v>34</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>35</v>
@@ -2815,11 +2906,13 @@
       <c r="G36" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H36" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H36" s="3"/>
+      <c r="I36" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J36" s="3"/>
+    </row>
+    <row r="37" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="13" t="s">
         <v>37</v>
       </c>
@@ -2830,7 +2923,7 @@
         <v>39</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>40</v>
@@ -2841,9 +2934,13 @@
       <c r="G37" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H37" s="7"/>
-    </row>
-    <row r="38" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H37" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="I37" s="7"/>
+      <c r="J37" s="7"/>
+    </row>
+    <row r="38" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="13" t="s">
         <v>42</v>
       </c>
@@ -2854,7 +2951,7 @@
         <v>44</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>45</v>
@@ -2865,11 +2962,13 @@
       <c r="G38" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H38" s="7" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H38" s="7"/>
+      <c r="I38" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="J38" s="7"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="14" t="s">
         <v>47</v>
       </c>
@@ -2880,7 +2979,7 @@
         <v>48</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>49</v>
@@ -2892,8 +2991,10 @@
         <v>319</v>
       </c>
       <c r="H39" s="3"/>
-    </row>
-    <row r="40" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+    </row>
+    <row r="40" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="13" t="s">
         <v>51</v>
       </c>
@@ -2904,7 +3005,7 @@
         <v>53</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>54</v>
@@ -2916,8 +3017,10 @@
         <v>319</v>
       </c>
       <c r="H40" s="7"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I40" s="7"/>
+      <c r="J40" s="7"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="14" t="s">
         <v>56</v>
       </c>
@@ -2928,7 +3031,7 @@
         <v>58</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>59</v>
@@ -2939,11 +3042,13 @@
       <c r="G41" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H41" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H41" s="3"/>
+      <c r="I41" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J41" s="3"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="14" t="s">
         <v>62</v>
       </c>
@@ -2954,7 +3059,7 @@
         <v>63</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>64</v>
@@ -2966,8 +3071,10 @@
         <v>319</v>
       </c>
       <c r="H42" s="3"/>
-    </row>
-    <row r="43" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+    </row>
+    <row r="43" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="13" t="s">
         <v>66</v>
       </c>
@@ -2978,7 +3085,7 @@
         <v>68</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>69</v>
@@ -2990,8 +3097,10 @@
         <v>319</v>
       </c>
       <c r="H43" s="7"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I43" s="7"/>
+      <c r="J43" s="7"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="14" t="s">
         <v>71</v>
       </c>
@@ -3002,7 +3111,7 @@
         <v>72</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>73</v>
@@ -3014,8 +3123,10 @@
         <v>319</v>
       </c>
       <c r="H44" s="3"/>
-    </row>
-    <row r="45" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+    </row>
+    <row r="45" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="13" t="s">
         <v>75</v>
       </c>
@@ -3026,7 +3137,7 @@
         <v>77</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>78</v>
@@ -3038,8 +3149,10 @@
         <v>319</v>
       </c>
       <c r="H45" s="7"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I45" s="7"/>
+      <c r="J45" s="7"/>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="14" t="s">
         <v>80</v>
       </c>
@@ -3050,7 +3163,7 @@
         <v>82</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>78</v>
@@ -3062,8 +3175,10 @@
         <v>319</v>
       </c>
       <c r="H46" s="3"/>
-    </row>
-    <row r="47" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
+    </row>
+    <row r="47" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="13" t="s">
         <v>84</v>
       </c>
@@ -3074,7 +3189,7 @@
         <v>86</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>87</v>
@@ -3085,11 +3200,15 @@
       <c r="G47" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H47" s="7" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H47" s="7"/>
+      <c r="I47" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="J47" s="7" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="14" t="s">
         <v>89</v>
       </c>
@@ -3100,7 +3219,7 @@
         <v>91</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>92</v>
@@ -3112,8 +3231,10 @@
         <v>319</v>
       </c>
       <c r="H48" s="3"/>
-    </row>
-    <row r="49" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+    </row>
+    <row r="49" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="13" t="s">
         <v>94</v>
       </c>
@@ -3124,7 +3245,7 @@
         <v>96</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>97</v>
@@ -3135,11 +3256,13 @@
       <c r="G49" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H49" s="7" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H49" s="7"/>
+      <c r="I49" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="J49" s="7"/>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="14" t="s">
         <v>99</v>
       </c>
@@ -3150,7 +3273,7 @@
         <v>101</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>78</v>
@@ -3162,8 +3285,12 @@
         <v>319</v>
       </c>
       <c r="H50" s="3"/>
-    </row>
-    <row r="51" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I50" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J50" s="3"/>
+    </row>
+    <row r="51" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="13" t="s">
         <v>103</v>
       </c>
@@ -3174,7 +3301,7 @@
         <v>105</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>106</v>
@@ -3186,8 +3313,10 @@
         <v>319</v>
       </c>
       <c r="H51" s="7"/>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I51" s="7"/>
+      <c r="J51" s="7"/>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="14" t="s">
         <v>108</v>
       </c>
@@ -3198,7 +3327,7 @@
         <v>110</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>111</v>
@@ -3210,8 +3339,10 @@
         <v>319</v>
       </c>
       <c r="H52" s="3"/>
-    </row>
-    <row r="53" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+    </row>
+    <row r="53" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="13" t="s">
         <v>113</v>
       </c>
@@ -3222,7 +3353,7 @@
         <v>114</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>115</v>
@@ -3234,8 +3365,10 @@
         <v>319</v>
       </c>
       <c r="H53" s="7"/>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I53" s="7"/>
+      <c r="J53" s="7"/>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="14" t="s">
         <v>117</v>
       </c>
@@ -3246,7 +3379,7 @@
         <v>119</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E54" s="3" t="s">
         <v>120</v>
@@ -3258,8 +3391,10 @@
         <v>319</v>
       </c>
       <c r="H54" s="3"/>
-    </row>
-    <row r="55" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+    </row>
+    <row r="55" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="13" t="s">
         <v>122</v>
       </c>
@@ -3270,7 +3405,7 @@
         <v>123</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>124</v>
@@ -3282,8 +3417,10 @@
         <v>319</v>
       </c>
       <c r="H55" s="7"/>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I55" s="7"/>
+      <c r="J55" s="7"/>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" s="14" t="s">
         <v>126</v>
       </c>
@@ -3294,7 +3431,7 @@
         <v>128</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E56" s="3" t="s">
         <v>129</v>
@@ -3305,11 +3442,13 @@
       <c r="G56" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H56" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H56" s="3"/>
+      <c r="I56" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J56" s="3"/>
+    </row>
+    <row r="57" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="13" t="s">
         <v>131</v>
       </c>
@@ -3320,7 +3459,7 @@
         <v>132</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>78</v>
@@ -3332,8 +3471,10 @@
         <v>319</v>
       </c>
       <c r="H57" s="7"/>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I57" s="7"/>
+      <c r="J57" s="7"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" s="14" t="s">
         <v>134</v>
       </c>
@@ -3344,7 +3485,7 @@
         <v>136</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>137</v>
@@ -3355,11 +3496,13 @@
       <c r="G58" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H58" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H58" s="3"/>
+      <c r="I58" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J58" s="3"/>
+    </row>
+    <row r="59" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="13" t="s">
         <v>139</v>
       </c>
@@ -3370,7 +3513,7 @@
         <v>141</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>142</v>
@@ -3381,9 +3524,13 @@
       <c r="G59" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H59" s="7"/>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H59" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="I59" s="7"/>
+      <c r="J59" s="7"/>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
         <v>144</v>
       </c>
@@ -3394,7 +3541,7 @@
         <v>145</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E60" s="3" t="s">
         <v>146</v>
@@ -3406,8 +3553,10 @@
         <v>319</v>
       </c>
       <c r="H60" s="3"/>
-    </row>
-    <row r="61" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I60" s="3"/>
+      <c r="J60" s="3"/>
+    </row>
+    <row r="61" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="13" t="s">
         <v>148</v>
       </c>
@@ -3418,7 +3567,7 @@
         <v>150</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>151</v>
@@ -3430,8 +3579,10 @@
         <v>319</v>
       </c>
       <c r="H61" s="7"/>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I61" s="7"/>
+      <c r="J61" s="7"/>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" s="14" t="s">
         <v>153</v>
       </c>
@@ -3442,7 +3593,7 @@
         <v>155</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>156</v>
@@ -3454,8 +3605,10 @@
         <v>319</v>
       </c>
       <c r="H62" s="3"/>
-    </row>
-    <row r="63" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I62" s="3"/>
+      <c r="J62" s="3"/>
+    </row>
+    <row r="63" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" s="13" t="s">
         <v>158</v>
       </c>
@@ -3466,7 +3619,7 @@
         <v>159</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>160</v>
@@ -3477,9 +3630,13 @@
       <c r="G63" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H63" s="7"/>
-    </row>
-    <row r="64" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H63" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="I63" s="7"/>
+      <c r="J63" s="7"/>
+    </row>
+    <row r="64" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" s="13" t="s">
         <v>162</v>
       </c>
@@ -3490,7 +3647,7 @@
         <v>164</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>165</v>
@@ -3502,8 +3659,10 @@
         <v>319</v>
       </c>
       <c r="H64" s="7"/>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I64" s="7"/>
+      <c r="J64" s="7"/>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="14" t="s">
         <v>167</v>
       </c>
@@ -3514,7 +3673,7 @@
         <v>169</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>170</v>
@@ -3526,8 +3685,10 @@
         <v>319</v>
       </c>
       <c r="H65" s="3"/>
-    </row>
-    <row r="66" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I65" s="3"/>
+      <c r="J65" s="3"/>
+    </row>
+    <row r="66" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="13" t="s">
         <v>172</v>
       </c>
@@ -3538,7 +3699,7 @@
         <v>174</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>175</v>
@@ -3550,8 +3711,10 @@
         <v>319</v>
       </c>
       <c r="H66" s="7"/>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I66" s="7"/>
+      <c r="J66" s="7"/>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="14" t="s">
         <v>177</v>
       </c>
@@ -3562,7 +3725,7 @@
         <v>179</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E67" s="3" t="s">
         <v>180</v>
@@ -3574,8 +3737,10 @@
         <v>319</v>
       </c>
       <c r="H67" s="3"/>
-    </row>
-    <row r="68" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I67" s="3"/>
+      <c r="J67" s="3"/>
+    </row>
+    <row r="68" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" s="13" t="s">
         <v>182</v>
       </c>
@@ -3586,7 +3751,7 @@
         <v>184</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>185</v>
@@ -3598,8 +3763,10 @@
         <v>319</v>
       </c>
       <c r="H68" s="7"/>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I68" s="7"/>
+      <c r="J68" s="7"/>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" s="14" t="s">
         <v>187</v>
       </c>
@@ -3610,7 +3777,7 @@
         <v>188</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>189</v>
@@ -3622,8 +3789,10 @@
         <v>319</v>
       </c>
       <c r="H69" s="3"/>
-    </row>
-    <row r="70" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I69" s="3"/>
+      <c r="J69" s="3"/>
+    </row>
+    <row r="70" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" s="13" t="s">
         <v>191</v>
       </c>
@@ -3634,7 +3803,7 @@
         <v>193</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>194</v>
@@ -3645,11 +3814,15 @@
       <c r="G70" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H70" s="7" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H70" s="7"/>
+      <c r="I70" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="J70" s="7" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" s="14" t="s">
         <v>196</v>
       </c>
@@ -3660,7 +3833,7 @@
         <v>198</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E71" s="8" t="s">
         <v>78</v>
@@ -3672,8 +3845,10 @@
         <v>319</v>
       </c>
       <c r="H71" s="3"/>
-    </row>
-    <row r="72" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I71" s="3"/>
+      <c r="J71" s="3"/>
+    </row>
+    <row r="72" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" s="13" t="s">
         <v>200</v>
       </c>
@@ -3684,7 +3859,7 @@
         <v>202</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>203</v>
@@ -3696,8 +3871,10 @@
         <v>319</v>
       </c>
       <c r="H72" s="7"/>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I72" s="7"/>
+      <c r="J72" s="7"/>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="14" t="s">
         <v>205</v>
       </c>
@@ -3708,7 +3885,7 @@
         <v>207</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E73" s="3"/>
       <c r="F73" s="5" t="s">
@@ -3718,8 +3895,10 @@
         <v>319</v>
       </c>
       <c r="H73" s="3"/>
-    </row>
-    <row r="74" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I73" s="3"/>
+      <c r="J73" s="3"/>
+    </row>
+    <row r="74" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A74" s="13" t="s">
         <v>209</v>
       </c>
@@ -3730,7 +3909,7 @@
         <v>211</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>212</v>
@@ -3741,9 +3920,13 @@
       <c r="G74" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H74" s="7"/>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H74" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="I74" s="7"/>
+      <c r="J74" s="7"/>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" s="14" t="s">
         <v>214</v>
       </c>
@@ -3754,7 +3937,7 @@
         <v>216</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E75" s="3"/>
       <c r="F75" s="5" t="s">
@@ -3764,8 +3947,10 @@
         <v>319</v>
       </c>
       <c r="H75" s="3"/>
-    </row>
-    <row r="76" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I75" s="3"/>
+      <c r="J75" s="3"/>
+    </row>
+    <row r="76" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" s="13" t="s">
         <v>218</v>
       </c>
@@ -3776,7 +3961,7 @@
         <v>219</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>220</v>
@@ -3787,9 +3972,13 @@
       <c r="G76" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H76" s="7"/>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H76" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="I76" s="7"/>
+      <c r="J76" s="7"/>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="14" t="s">
         <v>221</v>
       </c>
@@ -3800,7 +3989,7 @@
         <v>222</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E77" s="3" t="s">
         <v>223</v>
@@ -3811,11 +4000,13 @@
       <c r="G77" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H77" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="78" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H77" s="3"/>
+      <c r="I77" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J77" s="3"/>
+    </row>
+    <row r="78" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A78" s="13" t="s">
         <v>225</v>
       </c>
@@ -3826,7 +4017,7 @@
         <v>227</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>228</v>
@@ -3837,11 +4028,15 @@
       <c r="G78" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H78" s="7" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H78" s="7"/>
+      <c r="I78" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="J78" s="7" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" s="14" t="s">
         <v>230</v>
       </c>
@@ -3852,7 +4047,7 @@
         <v>232</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E79" s="3" t="s">
         <v>233</v>
@@ -3864,8 +4059,10 @@
         <v>319</v>
       </c>
       <c r="H79" s="3"/>
-    </row>
-    <row r="80" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I79" s="3"/>
+      <c r="J79" s="3"/>
+    </row>
+    <row r="80" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A80" s="13" t="s">
         <v>235</v>
       </c>
@@ -3876,7 +4073,7 @@
         <v>237</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>238</v>
@@ -3888,8 +4085,10 @@
         <v>319</v>
       </c>
       <c r="H80" s="7"/>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I80" s="7"/>
+      <c r="J80" s="7"/>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" s="14" t="s">
         <v>240</v>
       </c>
@@ -3900,7 +4099,7 @@
         <v>241</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E81" s="3" t="s">
         <v>242</v>
@@ -3911,11 +4110,13 @@
       <c r="G81" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H81" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H81" s="3"/>
+      <c r="I81" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J81" s="3"/>
+    </row>
+    <row r="82" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="13" t="s">
         <v>244</v>
       </c>
@@ -3926,7 +4127,7 @@
         <v>245</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E82" s="1" t="s">
         <v>246</v>
@@ -3938,8 +4139,10 @@
         <v>319</v>
       </c>
       <c r="H82" s="7"/>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I82" s="7"/>
+      <c r="J82" s="7"/>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" s="14" t="s">
         <v>248</v>
       </c>
@@ -3950,7 +4153,7 @@
         <v>250</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E83" s="3" t="s">
         <v>251</v>
@@ -3961,11 +4164,13 @@
       <c r="G83" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H83" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="84" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H83" s="3"/>
+      <c r="I83" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J83" s="3"/>
+    </row>
+    <row r="84" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A84" s="13" t="s">
         <v>253</v>
       </c>
@@ -3976,7 +4181,7 @@
         <v>255</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="E84" s="1" t="s">
         <v>256</v>
@@ -3988,8 +4193,10 @@
         <v>319</v>
       </c>
       <c r="H84" s="7"/>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I84" s="7"/>
+      <c r="J84" s="7"/>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" s="14" t="s">
         <v>258</v>
       </c>
@@ -4000,7 +4207,7 @@
         <v>259</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E85" s="3" t="s">
         <v>115</v>
@@ -4012,8 +4219,10 @@
         <v>319</v>
       </c>
       <c r="H85" s="3"/>
-    </row>
-    <row r="86" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I85" s="3"/>
+      <c r="J85" s="3"/>
+    </row>
+    <row r="86" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A86" s="13" t="s">
         <v>103</v>
       </c>
@@ -4024,7 +4233,7 @@
         <v>260</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E86" s="1" t="s">
         <v>106</v>
@@ -4036,8 +4245,10 @@
         <v>319</v>
       </c>
       <c r="H86" s="7"/>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I86" s="7"/>
+      <c r="J86" s="7"/>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" s="14" t="s">
         <v>261</v>
       </c>
@@ -4048,7 +4259,7 @@
         <v>262</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E87" s="3" t="s">
         <v>263</v>
@@ -4060,8 +4271,10 @@
         <v>319</v>
       </c>
       <c r="H87" s="3"/>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I87" s="3"/>
+      <c r="J87" s="3"/>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" s="14" t="s">
         <v>266</v>
       </c>
@@ -4072,7 +4285,7 @@
         <v>268</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E88" s="3" t="s">
         <v>269</v>
@@ -4084,8 +4297,10 @@
         <v>319</v>
       </c>
       <c r="H88" s="3"/>
-    </row>
-    <row r="89" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I88" s="3"/>
+      <c r="J88" s="3"/>
+    </row>
+    <row r="89" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A89" s="13" t="s">
         <v>271</v>
       </c>
@@ -4096,7 +4311,7 @@
         <v>272</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E89" s="1" t="s">
         <v>273</v>
@@ -4107,9 +4322,13 @@
       <c r="G89" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H89" s="7"/>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H89" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="I89" s="7"/>
+      <c r="J89" s="7"/>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" s="14" t="s">
         <v>275</v>
       </c>
@@ -4120,7 +4339,7 @@
         <v>277</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E90" s="3" t="s">
         <v>278</v>
@@ -4132,8 +4351,10 @@
         <v>319</v>
       </c>
       <c r="H90" s="3"/>
-    </row>
-    <row r="91" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I90" s="3"/>
+      <c r="J90" s="3"/>
+    </row>
+    <row r="91" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A91" s="13" t="s">
         <v>280</v>
       </c>
@@ -4144,7 +4365,7 @@
         <v>281</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E91" s="1" t="s">
         <v>282</v>
@@ -4155,22 +4376,24 @@
       <c r="G91" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H91" s="7" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H91" s="7"/>
+      <c r="I91" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="J91" s="7"/>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" s="14" t="s">
         <v>284</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C92" s="18" t="s">
         <v>285</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>286</v>
@@ -4181,11 +4404,13 @@
       <c r="G92" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H92" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="93" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H92" s="3"/>
+      <c r="I92" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J92" s="3"/>
+    </row>
+    <row r="93" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A93" s="13" t="s">
         <v>182</v>
       </c>
@@ -4196,7 +4421,7 @@
         <v>184</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="E93" s="1" t="s">
         <v>185</v>
@@ -4208,8 +4433,10 @@
         <v>319</v>
       </c>
       <c r="H93" s="7"/>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I93" s="7"/>
+      <c r="J93" s="7"/>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" s="14" t="s">
         <v>288</v>
       </c>
@@ -4220,7 +4447,7 @@
         <v>289</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E94" s="3" t="s">
         <v>290</v>
@@ -4232,8 +4459,10 @@
         <v>319</v>
       </c>
       <c r="H94" s="3"/>
-    </row>
-    <row r="95" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I94" s="3"/>
+      <c r="J94" s="3"/>
+    </row>
+    <row r="95" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A95" s="13" t="s">
         <v>292</v>
       </c>
@@ -4244,7 +4473,7 @@
         <v>294</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E95" s="1" t="s">
         <v>295</v>
@@ -4256,19 +4485,21 @@
         <v>319</v>
       </c>
       <c r="H95" s="7"/>
-    </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I95" s="7"/>
+      <c r="J95" s="7"/>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96" s="14" t="s">
         <v>297</v>
       </c>
       <c r="B96" s="19" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C96" s="18" t="s">
         <v>298</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E96" s="3" t="s">
         <v>299</v>
@@ -4280,8 +4511,10 @@
         <v>319</v>
       </c>
       <c r="H96" s="3"/>
-    </row>
-    <row r="97" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I96" s="3"/>
+      <c r="J96" s="3"/>
+    </row>
+    <row r="97" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A97" s="13" t="s">
         <v>301</v>
       </c>
@@ -4292,7 +4525,7 @@
         <v>303</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E97" s="1" t="s">
         <v>304</v>
@@ -4304,8 +4537,10 @@
         <v>319</v>
       </c>
       <c r="H97" s="7"/>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I97" s="7"/>
+      <c r="J97" s="7"/>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98" s="14" t="s">
         <v>306</v>
       </c>
@@ -4316,7 +4551,7 @@
         <v>307</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E98" s="3" t="s">
         <v>308</v>
@@ -4327,22 +4562,24 @@
       <c r="G98" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H98" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="99" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H98" s="3"/>
+      <c r="I98" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J98" s="3"/>
+    </row>
+    <row r="99" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A99" s="13" t="s">
         <v>310</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C99" s="17" t="s">
         <v>311</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E99" s="1" t="s">
         <v>312</v>
@@ -4354,8 +4591,10 @@
         <v>319</v>
       </c>
       <c r="H99" s="7"/>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I99" s="7"/>
+      <c r="J99" s="7"/>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" s="14" t="s">
         <v>314</v>
       </c>
@@ -4366,7 +4605,7 @@
         <v>316</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E100" s="3" t="s">
         <v>317</v>
@@ -4377,11 +4616,15 @@
       <c r="G100" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H100" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="101" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H100" s="3"/>
+      <c r="I100" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="J100" s="3" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A101" s="15" t="s">
         <v>321</v>
       </c>
@@ -4392,7 +4635,7 @@
         <v>323</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E101" s="1" t="s">
         <v>324</v>
@@ -4404,8 +4647,10 @@
         <v>319</v>
       </c>
       <c r="H101" s="7"/>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I101" s="7"/>
+      <c r="J101" s="7"/>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A102" s="16" t="s">
         <v>326</v>
       </c>
@@ -4416,7 +4661,7 @@
         <v>327</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E102" s="3" t="s">
         <v>328</v>
@@ -4427,9 +4672,13 @@
       <c r="G102" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="H102" s="3"/>
-    </row>
-    <row r="103" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H102" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="I102" s="3"/>
+      <c r="J102" s="3"/>
+    </row>
+    <row r="103" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A103" s="15" t="s">
         <v>330</v>
       </c>
@@ -4440,7 +4689,7 @@
         <v>332</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E103" s="1" t="s">
         <v>333</v>
@@ -4451,11 +4700,13 @@
       <c r="G103" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="H103" s="7" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H103" s="7"/>
+      <c r="I103" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="J103" s="7"/>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A104" s="16" t="s">
         <v>335</v>
       </c>
@@ -4466,7 +4717,7 @@
         <v>337</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E104" s="3" t="s">
         <v>338</v>
@@ -4478,8 +4729,10 @@
         <v>319</v>
       </c>
       <c r="H104" s="3"/>
-    </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I104" s="3"/>
+      <c r="J104" s="3"/>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A105" s="15" t="s">
         <v>340</v>
       </c>
@@ -4490,7 +4743,7 @@
         <v>341</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E105" s="1" t="s">
         <v>342</v>
@@ -4502,8 +4755,10 @@
         <v>319</v>
       </c>
       <c r="H105" s="1"/>
-    </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I105" s="1"/>
+      <c r="J105" s="1"/>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A106" s="16" t="s">
         <v>344</v>
       </c>
@@ -4514,7 +4769,7 @@
         <v>345</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E106" s="3" t="s">
         <v>346</v>
@@ -4526,11 +4781,13 @@
         <v>319</v>
       </c>
       <c r="H106" s="3"/>
+      <c r="I106" s="3"/>
+      <c r="J106" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C29" r:id="rId1" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>

</xml_diff>